<commit_message>
Medalists UI: split All row, teal/slate filters, equal mode buttons
- medals.html: T1 All on own row; T2 Individual/Pairs/Teams; fix panel JS
- style.css: medal filter pills, .medal-panel[hidden], equal-width mode buttons
- rank.xlsx: name normalizations (from prior edits in working tree)
- team_results: Johnny/Kare team name spelling (ovako, sova)
</commit_message>
<xml_diff>
--- a/rank.xlsx
+++ b/rank.xlsx
@@ -1749,7 +1749,7 @@
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>Gvido Piasevoli</t>
+          <t>Guido Piasevoli</t>
         </is>
       </c>
       <c r="C67" s="1" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="B105" s="1" t="inlineStr">
         <is>
-          <t>Gvido Piasevoli</t>
+          <t>Guido Piasevoli</t>
         </is>
       </c>
       <c r="C105" s="1" t="n">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="B110" s="1" t="inlineStr">
         <is>
-          <t>Ivan Požežanac-Hajić</t>
+          <t>Ivan Požežanac Hajić</t>
         </is>
       </c>
       <c r="C110" s="1" t="n">
@@ -8082,7 +8082,7 @@
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>Davor Požežanac-Hajić</t>
+          <t>Davor Požežanac Hajić</t>
         </is>
       </c>
       <c r="C121" s="1" t="n">
@@ -8212,7 +8212,7 @@
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>Gvido Piasevoli</t>
+          <t>Guido Piasevoli</t>
         </is>
       </c>
       <c r="C131" s="1" t="n">
@@ -10597,7 +10597,7 @@
       </c>
       <c r="B88" s="1" t="inlineStr">
         <is>
-          <t>Ivan Požežanac-Hajić</t>
+          <t>Ivan Požežanac Hajić</t>
         </is>
       </c>
       <c r="C88" s="1" t="n">
@@ -10844,7 +10844,7 @@
       </c>
       <c r="B107" s="1" t="inlineStr">
         <is>
-          <t>Gvido Piasevoli</t>
+          <t>Guido Piasevoli</t>
         </is>
       </c>
       <c r="C107" s="1" t="n">
@@ -12983,7 +12983,7 @@
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t>Ivan Covic</t>
+          <t>Ivan Čović</t>
         </is>
       </c>
       <c r="C40" s="1" t="n">
@@ -13555,7 +13555,7 @@
       </c>
       <c r="B84" s="1" t="inlineStr">
         <is>
-          <t>Ivan Požežanac-Hajić</t>
+          <t>Ivan Požežanac Hajić</t>
         </is>
       </c>
       <c r="C84" s="1" t="n">
@@ -13581,7 +13581,7 @@
       </c>
       <c r="B86" s="1" t="inlineStr">
         <is>
-          <t>Slobodan Pavlovic</t>
+          <t>Slobodan Pavlović</t>
         </is>
       </c>
       <c r="C86" s="1" t="n">
@@ -14010,7 +14010,7 @@
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>Matko Dujmovic</t>
+          <t>Matko Dujmović</t>
         </is>
       </c>
       <c r="C119" s="1" t="n">
@@ -14023,7 +14023,7 @@
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>Gvido Piasevoli</t>
+          <t>Guido Piasevoli</t>
         </is>
       </c>
       <c r="C120" s="1" t="n">
@@ -14088,7 +14088,7 @@
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>Arandjel Smiljanic</t>
+          <t>Aranđel Smiljanić</t>
         </is>
       </c>
       <c r="C125" s="1" t="n">
@@ -14270,7 +14270,7 @@
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>Mislav Ivankovic</t>
+          <t>Mislav Ivanković</t>
         </is>
       </c>
       <c r="C139" s="1" t="n">
@@ -14595,7 +14595,7 @@
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>Goran Djaković</t>
+          <t>Goran Đaković</t>
         </is>
       </c>
       <c r="C164" s="1" t="n">
@@ -16385,7 +16385,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Ivan Požežanac</t>
+          <t>Ivan Požežanac Hajić</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -17303,7 +17303,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Ivan Požežanac</t>
+          <t>Ivan Požežanac Hajić</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -19001,7 +19001,7 @@
       </c>
       <c r="B101" s="1" t="inlineStr">
         <is>
-          <t>Ivan Požežanac</t>
+          <t>Ivan Požežanac Hajić</t>
         </is>
       </c>
       <c r="C101" s="1" t="n">
@@ -19872,7 +19872,7 @@
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>Gvido Piasevoli</t>
+          <t>Guido Piasevoli</t>
         </is>
       </c>
       <c r="C168" s="1" t="n">
@@ -19950,7 +19950,7 @@
       </c>
       <c r="B174" s="1" t="inlineStr">
         <is>
-          <t>Arandjel Smiljanić</t>
+          <t>Aranđel Smiljanić</t>
         </is>
       </c>
       <c r="C174" s="1" t="n">
@@ -23188,7 +23188,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Ivan Požežanac</t>
+          <t>Ivan Požežanac Hajić</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -23292,7 +23292,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Marko Poličič</t>
+          <t>Marko Poličić</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -23630,7 +23630,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Marijan Pandzic</t>
+          <t>Marijan Pandžić</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -24571,7 +24571,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Gvido Piasevoli</t>
+          <t>Guido Piasevoli</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -25946,7 +25946,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Gvido Piasevoli</t>
+          <t>Guido Piasevoli</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -26461,7 +26461,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Dino Milić - Jakovlić</t>
+          <t>Dino Milić-Jakovlić</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -28468,7 +28468,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Gvido Piasevoli</t>
+          <t>Guido Piasevoli</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -28637,7 +28637,7 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Tino Nevešćanin</t>
+          <t>Tino Neveščanin</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -31824,7 +31824,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Gvido Piasevoli</t>
+          <t>Guido Piasevoli</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -32998,7 +32998,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Tino Nevešćanin</t>
+          <t>Tino Neveščanin</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -33735,7 +33735,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Ivan Požežanac</t>
+          <t>Ivan Požežanac Hajić</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -35210,7 +35210,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Jasmin MIkolčević</t>
+          <t>Jasmin Mikolčević</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Nikola Pezic</t>
+          <t>Nikola Pezić</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
@@ -36401,7 +36401,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Dino Milić - Jakovlić</t>
+          <t>Dino Milić-Jakovlić</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -36518,7 +36518,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Tomislav Curin</t>
+          <t>Tomislav Ćurin</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
@@ -36531,7 +36531,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Mirko Miocic</t>
+          <t>Mirko Miočić</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -36622,7 +36622,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Mario Marušic</t>
+          <t>Mario Marušić</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
@@ -36726,7 +36726,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Ankica Vukelic</t>
+          <t>Ankica Vukelić</t>
         </is>
       </c>
       <c r="C36" s="3" t="n">
@@ -36752,7 +36752,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Emiljana Vozila mohorović</t>
+          <t>Emiljana Vozila Mohorović</t>
         </is>
       </c>
       <c r="C38" s="3" t="n">
@@ -36869,7 +36869,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Zoran Mikovic</t>
+          <t>Zoran Miković</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
@@ -36960,7 +36960,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Snjezana Buncic</t>
+          <t>Snježana Bunčić</t>
         </is>
       </c>
       <c r="C54" s="3" t="n">
@@ -36973,7 +36973,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Alen Barbic</t>
+          <t>Alen Barbić</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
@@ -37012,7 +37012,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Ivana Kurecic</t>
+          <t>Ivana Kurečić</t>
         </is>
       </c>
       <c r="C58" s="3" t="n">
@@ -37038,7 +37038,7 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Franjo-Josip Markovic</t>
+          <t>Franjo-Josip Marković</t>
         </is>
       </c>
       <c r="C60" s="3" t="n">
@@ -37433,7 +37433,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Dino Milić - Jakovlić</t>
+          <t>Dino Milić-Jakovlić</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
@@ -38894,7 +38894,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Dino Milić - Jakovlić</t>
+          <t>Dino Milić-Jakovlić</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
@@ -39939,7 +39939,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Dino Milić - Jakovlić</t>
+          <t>Dino Milić-Jakovlić</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
@@ -40251,7 +40251,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Nikola Delic</t>
+          <t>Nikola Delić</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
@@ -41205,7 +41205,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Dino Milić - Jakovlić</t>
+          <t>Dino Milić-Jakovlić</t>
         </is>
       </c>
       <c r="C30" s="3" t="n">
@@ -41725,7 +41725,7 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Emiljana Vozila mohorović</t>
+          <t>Emiljana Vozila Mohorović</t>
         </is>
       </c>
       <c r="C70" s="3" t="n">
@@ -42575,7 +42575,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Nikola Pezic</t>
+          <t>Nikola Pezić</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -42679,7 +42679,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Dino Milić - Jakovlić</t>
+          <t>Dino Milić-Jakovlić</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
@@ -42809,7 +42809,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Dario Pejin</t>
+          <t>Darijo Pejin</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
@@ -43854,7 +43854,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Ivan Požežanac</t>
+          <t>Ivan Požežanac Hajić</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -43932,7 +43932,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Dino Milić - Jakovlić</t>
+          <t>Dino Milić-Jakovlić</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
@@ -45016,7 +45016,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Dario Butkovic</t>
+          <t>Dario Butković</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
@@ -45029,7 +45029,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Dino Milić - Jakovlić</t>
+          <t>Dino Milić-Jakovlić</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
@@ -45601,7 +45601,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Nikola Delic</t>
+          <t>Nikola Delić</t>
         </is>
       </c>
       <c r="C72" s="3" t="n">
@@ -45692,7 +45692,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Danijel Letica</t>
+          <t>Daniel Letica</t>
         </is>
       </c>
       <c r="C79" s="3" t="n">
@@ -45757,7 +45757,7 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Andrej Plećaš</t>
+          <t>Andrej Plečaš</t>
         </is>
       </c>
       <c r="C84" s="3" t="n">
@@ -45978,7 +45978,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Emiljana Vozila mohorović</t>
+          <t>Emiljana Vozila Mohorović</t>
         </is>
       </c>
       <c r="C101" s="3" t="n">
@@ -46524,7 +46524,7 @@
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>Roc Stilinovic</t>
+          <t>Roč Stilinović</t>
         </is>
       </c>
       <c r="C143" s="3" t="n">
@@ -47439,7 +47439,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Dino Milić - Jakovlić</t>
+          <t>Dino Milić-Jakovlić</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
@@ -47920,7 +47920,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Dario Pejin</t>
+          <t>Darijo Pejin</t>
         </is>
       </c>
       <c r="C76" s="3" t="n">
@@ -47933,7 +47933,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Nikola Delic</t>
+          <t>Nikola Delić</t>
         </is>
       </c>
       <c r="C77" s="3" t="n">
@@ -48037,7 +48037,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Emiljana Vozila mohorović</t>
+          <t>Emiljana Vozila Mohorović</t>
         </is>
       </c>
       <c r="C85" s="3" t="n">
@@ -48297,7 +48297,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Božidar Marjanovic</t>
+          <t>Božidar Marjanović</t>
         </is>
       </c>
       <c r="C105" s="3" t="n">
@@ -48960,7 +48960,7 @@
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>Ivan Tomic</t>
+          <t>Ivan Tomić</t>
         </is>
       </c>
       <c r="C156" s="3" t="n">
@@ -52379,7 +52379,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Danijel Letica</t>
+          <t>Daniel Letica</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
@@ -52600,7 +52600,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Božidar Marjanovic</t>
+          <t>Božidar Marjanović</t>
         </is>
       </c>
       <c r="C46" s="3" t="n">
@@ -53003,7 +53003,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Emiljana Vozila mohorović</t>
+          <t>Emiljana Vozila Mohorović</t>
         </is>
       </c>
       <c r="C77" s="3" t="n">
@@ -53263,7 +53263,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Zoran Mikovic</t>
+          <t>Zoran Miković</t>
         </is>
       </c>
       <c r="C97" s="3" t="n">
@@ -53289,7 +53289,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Ivan Tomic</t>
+          <t>Ivan Tomić</t>
         </is>
       </c>
       <c r="C99" s="3" t="n">
@@ -53497,7 +53497,7 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Roc Stilinovic</t>
+          <t>Roč Stilinović</t>
         </is>
       </c>
       <c r="C115" s="3" t="n">
@@ -53523,7 +53523,7 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Ðuro Jurišić</t>
+          <t>Đuro Jurišić</t>
         </is>
       </c>
       <c r="C117" s="3" t="n">
@@ -53892,7 +53892,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Dino Milić - Jakovlić</t>
+          <t>Dino Milić-Jakovlić</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
@@ -53931,7 +53931,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Danijel Letica</t>
+          <t>Daniel Letica</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
@@ -53970,7 +53970,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Emilijana Vozila Mohorovic</t>
+          <t>Emiljana Vozila Mohorović</t>
         </is>
       </c>
       <c r="C32" s="3" t="n">
@@ -53983,7 +53983,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Mislav Zuanovic</t>
+          <t>Mislav Zuanović</t>
         </is>
       </c>
       <c r="C33" s="3" t="n">
@@ -54243,7 +54243,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Ankica Vukelic</t>
+          <t>Ankica Vukelić</t>
         </is>
       </c>
       <c r="C53" s="3" t="n">
@@ -54256,7 +54256,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Željko Šilovic</t>
+          <t>Željko Šilović</t>
         </is>
       </c>
       <c r="C54" s="3" t="n">
@@ -54269,7 +54269,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Mario Brkic</t>
+          <t>Mario Brkić</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
@@ -54347,7 +54347,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Ante Maric</t>
+          <t>Ante Marić</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
@@ -54412,7 +54412,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Ivan Tomic</t>
+          <t>Ivan Tomić</t>
         </is>
       </c>
       <c r="C66" s="3" t="n">
@@ -54438,7 +54438,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Goran Bjelic</t>
+          <t>Goran Bjelić</t>
         </is>
       </c>
       <c r="C68" s="3" t="n">
@@ -54451,7 +54451,7 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Luka Pamic</t>
+          <t>Luka Pamić</t>
         </is>
       </c>
       <c r="C69" s="3" t="n">
@@ -54477,7 +54477,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Roc Stilinovic</t>
+          <t>Roč Stilinović</t>
         </is>
       </c>
       <c r="C71" s="3" t="n">
@@ -54490,7 +54490,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Haris Zubcevic</t>
+          <t>Haris Zubčević</t>
         </is>
       </c>
       <c r="C72" s="3" t="n">
@@ -54503,7 +54503,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Filip Milkovic</t>
+          <t>Filip Milković</t>
         </is>
       </c>
       <c r="C73" s="3" t="n">
@@ -54516,7 +54516,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Jasminka Piralic</t>
+          <t>Jasminka Piralić</t>
         </is>
       </c>
       <c r="C74" s="3" t="n">
@@ -54542,7 +54542,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Krešimir Šimic</t>
+          <t>Krešimir Šimić</t>
         </is>
       </c>
       <c r="C76" s="3" t="n">
@@ -54568,7 +54568,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>David Condic</t>
+          <t>David Čondić</t>
         </is>
       </c>
       <c r="C78" s="3" t="n">
@@ -54581,7 +54581,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Marin Zupicic</t>
+          <t>Marin Župičić</t>
         </is>
       </c>
       <c r="C79" s="3" t="n">
@@ -56179,7 +56179,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Tomy Kunović</t>
+          <t>Tomi Kunović</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -56744,7 +56744,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Boris Bečić</t>
+          <t>Boris Benčić</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -57971,7 +57971,7 @@
       </c>
       <c r="B79" s="1" t="inlineStr">
         <is>
-          <t>Gvido Piasevoli</t>
+          <t>Guido Piasevoli</t>
         </is>
       </c>
       <c r="C79" s="1" t="n">

</xml_diff>

<commit_message>
feat: add SOVA 2026
</commit_message>
<xml_diff>
--- a/rank.xlsx
+++ b/rank.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neven/Documents/github-repos/croatian-quiz-scores/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63F74BC4-E0FD-A84D-B7B1-A6C471EC5BC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04899E9C-A298-BC4E-A854-15F0F82684FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19220" firstSheet="16" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,29 +33,30 @@
     <sheet name="SOVA 2025" sheetId="18" r:id="rId18"/>
     <sheet name="MMM 2025" sheetId="19" r:id="rId19"/>
     <sheet name="Osijek Open 2025" sheetId="20" r:id="rId20"/>
-    <sheet name="Croatian Open 2015" sheetId="44" r:id="rId21"/>
-    <sheet name="Croatian Open 2016" sheetId="45" r:id="rId22"/>
-    <sheet name="Croatian Open 2017" sheetId="21" r:id="rId23"/>
-    <sheet name="Croatian Open 2018" sheetId="22" r:id="rId24"/>
-    <sheet name="Croatian Open 2019" sheetId="23" r:id="rId25"/>
-    <sheet name="Croatian Open 2020" sheetId="24" r:id="rId26"/>
-    <sheet name="Croatian Open 2021" sheetId="25" r:id="rId27"/>
-    <sheet name="Croatian Open 2022" sheetId="26" r:id="rId28"/>
-    <sheet name="Croatian Open 2023" sheetId="27" r:id="rId29"/>
-    <sheet name="Croatian Open 2024" sheetId="28" r:id="rId30"/>
-    <sheet name="Croatian Open 2025" sheetId="29" r:id="rId31"/>
-    <sheet name="WQC 2014" sheetId="30" r:id="rId32"/>
-    <sheet name="WQC 2015" sheetId="31" r:id="rId33"/>
-    <sheet name="WQC 2025" sheetId="32" r:id="rId34"/>
-    <sheet name="WQC 2024" sheetId="33" r:id="rId35"/>
-    <sheet name="WQC 2023" sheetId="34" r:id="rId36"/>
-    <sheet name="WQC 2022" sheetId="35" r:id="rId37"/>
-    <sheet name="WQC 2021" sheetId="36" r:id="rId38"/>
-    <sheet name="WQC 2020" sheetId="37" r:id="rId39"/>
-    <sheet name="WQC 2019" sheetId="38" r:id="rId40"/>
-    <sheet name="WQC 2018" sheetId="39" r:id="rId41"/>
-    <sheet name="WQC 2017" sheetId="40" r:id="rId42"/>
-    <sheet name="WQC 2016" sheetId="41" r:id="rId43"/>
+    <sheet name="SOVA 2026" sheetId="46" r:id="rId21"/>
+    <sheet name="Croatian Open 2015" sheetId="44" r:id="rId22"/>
+    <sheet name="Croatian Open 2016" sheetId="45" r:id="rId23"/>
+    <sheet name="Croatian Open 2017" sheetId="21" r:id="rId24"/>
+    <sheet name="Croatian Open 2018" sheetId="22" r:id="rId25"/>
+    <sheet name="Croatian Open 2019" sheetId="23" r:id="rId26"/>
+    <sheet name="Croatian Open 2020" sheetId="24" r:id="rId27"/>
+    <sheet name="Croatian Open 2021" sheetId="25" r:id="rId28"/>
+    <sheet name="Croatian Open 2022" sheetId="26" r:id="rId29"/>
+    <sheet name="Croatian Open 2023" sheetId="27" r:id="rId30"/>
+    <sheet name="Croatian Open 2024" sheetId="28" r:id="rId31"/>
+    <sheet name="Croatian Open 2025" sheetId="29" r:id="rId32"/>
+    <sheet name="WQC 2014" sheetId="30" r:id="rId33"/>
+    <sheet name="WQC 2015" sheetId="31" r:id="rId34"/>
+    <sheet name="WQC 2025" sheetId="32" r:id="rId35"/>
+    <sheet name="WQC 2024" sheetId="33" r:id="rId36"/>
+    <sheet name="WQC 2023" sheetId="34" r:id="rId37"/>
+    <sheet name="WQC 2022" sheetId="35" r:id="rId38"/>
+    <sheet name="WQC 2021" sheetId="36" r:id="rId39"/>
+    <sheet name="WQC 2020" sheetId="37" r:id="rId40"/>
+    <sheet name="WQC 2019" sheetId="38" r:id="rId41"/>
+    <sheet name="WQC 2018" sheetId="39" r:id="rId42"/>
+    <sheet name="WQC 2017" sheetId="40" r:id="rId43"/>
+    <sheet name="WQC 2016" sheetId="41" r:id="rId44"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -74,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4036" uniqueCount="931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4135" uniqueCount="947">
   <si>
     <t>Krešimir Štimac</t>
   </si>
@@ -2867,6 +2868,54 @@
   </si>
   <si>
     <t>Grgur Erak</t>
+  </si>
+  <si>
+    <t>Domagoj Šobatović</t>
+  </si>
+  <si>
+    <t>Marijan Smodlaka</t>
+  </si>
+  <si>
+    <t>Paško Sorić</t>
+  </si>
+  <si>
+    <t>Ivan Požežanac</t>
+  </si>
+  <si>
+    <t>Rene Benić</t>
+  </si>
+  <si>
+    <t>Bernard Pervan</t>
+  </si>
+  <si>
+    <t>Ivan Livančić</t>
+  </si>
+  <si>
+    <t>Dario Ćorić</t>
+  </si>
+  <si>
+    <t>Emir Džaferović</t>
+  </si>
+  <si>
+    <t>Leira Harabalja</t>
+  </si>
+  <si>
+    <t>Tin Šimunić</t>
+  </si>
+  <si>
+    <t>Goran Šantak</t>
+  </si>
+  <si>
+    <t>Ivica Tomljanović</t>
+  </si>
+  <si>
+    <t>Dario Matešić</t>
+  </si>
+  <si>
+    <t>Jure Lubina</t>
+  </si>
+  <si>
+    <t>Filip Špoljarić</t>
   </si>
 </sst>
 </file>
@@ -23861,6 +23910,1135 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FF75AEB-59E2-CF45-BBD9-3E4062C7B61F}">
+  <dimension ref="A1:D99"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C1">
+        <v>153</v>
+      </c>
+      <c r="D1">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2">
+        <v>148</v>
+      </c>
+      <c r="D2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3">
+        <v>148</v>
+      </c>
+      <c r="D3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>275</v>
+      </c>
+      <c r="C4">
+        <v>143</v>
+      </c>
+      <c r="D4">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C5">
+        <v>141</v>
+      </c>
+      <c r="D5">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>295</v>
+      </c>
+      <c r="C6">
+        <v>139</v>
+      </c>
+      <c r="D6">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>260</v>
+      </c>
+      <c r="C7">
+        <v>137</v>
+      </c>
+      <c r="D7">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C8">
+        <v>136</v>
+      </c>
+      <c r="D8">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>342</v>
+      </c>
+      <c r="C9">
+        <v>135</v>
+      </c>
+      <c r="D9">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>931</v>
+      </c>
+      <c r="C10">
+        <v>131</v>
+      </c>
+      <c r="D10">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>127</v>
+      </c>
+      <c r="C13">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>932</v>
+      </c>
+      <c r="C14">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>351</v>
+      </c>
+      <c r="C15">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>310</v>
+      </c>
+      <c r="C16">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>352</v>
+      </c>
+      <c r="C17">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>18</v>
+      </c>
+      <c r="B18" t="s">
+        <v>391</v>
+      </c>
+      <c r="C18">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>21</v>
+      </c>
+      <c r="B21" t="s">
+        <v>140</v>
+      </c>
+      <c r="C21">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>302</v>
+      </c>
+      <c r="C22">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>23</v>
+      </c>
+      <c r="B23" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>24</v>
+      </c>
+      <c r="B24" t="s">
+        <v>659</v>
+      </c>
+      <c r="C24">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>3</v>
+      </c>
+      <c r="C25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
+        <v>382</v>
+      </c>
+      <c r="C26">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>27</v>
+      </c>
+      <c r="B27" t="s">
+        <v>503</v>
+      </c>
+      <c r="C27">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>508</v>
+      </c>
+      <c r="C28">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>27</v>
+      </c>
+      <c r="B29" t="s">
+        <v>933</v>
+      </c>
+      <c r="C29">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>30</v>
+      </c>
+      <c r="B30" t="s">
+        <v>279</v>
+      </c>
+      <c r="C30">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>507</v>
+      </c>
+      <c r="C31">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>32</v>
+      </c>
+      <c r="B32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C32">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>51</v>
+      </c>
+      <c r="C33">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>34</v>
+      </c>
+      <c r="B34" t="s">
+        <v>277</v>
+      </c>
+      <c r="C34">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>473</v>
+      </c>
+      <c r="C35">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>34</v>
+      </c>
+      <c r="B36" t="s">
+        <v>259</v>
+      </c>
+      <c r="C36">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>34</v>
+      </c>
+      <c r="B37" t="s">
+        <v>300</v>
+      </c>
+      <c r="C37">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>34</v>
+      </c>
+      <c r="B38" t="s">
+        <v>303</v>
+      </c>
+      <c r="C38">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>34</v>
+      </c>
+      <c r="B39" t="s">
+        <v>427</v>
+      </c>
+      <c r="C39">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>40</v>
+      </c>
+      <c r="B40" t="s">
+        <v>511</v>
+      </c>
+      <c r="C40">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>55</v>
+      </c>
+      <c r="C41">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>40</v>
+      </c>
+      <c r="B42" t="s">
+        <v>314</v>
+      </c>
+      <c r="C42">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>43</v>
+      </c>
+      <c r="B43" t="s">
+        <v>308</v>
+      </c>
+      <c r="C43">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>45</v>
+      </c>
+      <c r="B45" t="s">
+        <v>484</v>
+      </c>
+      <c r="C45">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>46</v>
+      </c>
+      <c r="B46" t="s">
+        <v>26</v>
+      </c>
+      <c r="C46">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>47</v>
+      </c>
+      <c r="B47" t="s">
+        <v>518</v>
+      </c>
+      <c r="C47">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>934</v>
+      </c>
+      <c r="C48">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>47</v>
+      </c>
+      <c r="B49" t="s">
+        <v>935</v>
+      </c>
+      <c r="C49">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>50</v>
+      </c>
+      <c r="B50" t="s">
+        <v>537</v>
+      </c>
+      <c r="C50">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>51</v>
+      </c>
+      <c r="B51" t="s">
+        <v>316</v>
+      </c>
+      <c r="C51">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>401</v>
+      </c>
+      <c r="C52">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>53</v>
+      </c>
+      <c r="B53" t="s">
+        <v>936</v>
+      </c>
+      <c r="C53">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>521</v>
+      </c>
+      <c r="C54">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>53</v>
+      </c>
+      <c r="B55" t="s">
+        <v>22</v>
+      </c>
+      <c r="C55">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>53</v>
+      </c>
+      <c r="B56" t="s">
+        <v>470</v>
+      </c>
+      <c r="C56">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>57</v>
+      </c>
+      <c r="B57" t="s">
+        <v>527</v>
+      </c>
+      <c r="C57">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>223</v>
+      </c>
+      <c r="C58">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>59</v>
+      </c>
+      <c r="B59" t="s">
+        <v>937</v>
+      </c>
+      <c r="C59">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>446</v>
+      </c>
+      <c r="C60">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61">
+        <v>59</v>
+      </c>
+      <c r="B61" t="s">
+        <v>435</v>
+      </c>
+      <c r="C61">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62">
+        <v>62</v>
+      </c>
+      <c r="B62" t="s">
+        <v>489</v>
+      </c>
+      <c r="C62">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>284</v>
+      </c>
+      <c r="C63">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64">
+        <v>64</v>
+      </c>
+      <c r="B64" t="s">
+        <v>513</v>
+      </c>
+      <c r="C64">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>357</v>
+      </c>
+      <c r="C65">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>64</v>
+      </c>
+      <c r="B66" t="s">
+        <v>433</v>
+      </c>
+      <c r="C66">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>67</v>
+      </c>
+      <c r="B67" t="s">
+        <v>531</v>
+      </c>
+      <c r="C67">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>488</v>
+      </c>
+      <c r="C68">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>67</v>
+      </c>
+      <c r="B69" t="s">
+        <v>542</v>
+      </c>
+      <c r="C69">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>67</v>
+      </c>
+      <c r="B70" t="s">
+        <v>440</v>
+      </c>
+      <c r="C70">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>71</v>
+      </c>
+      <c r="B71" t="s">
+        <v>486</v>
+      </c>
+      <c r="C71">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>324</v>
+      </c>
+      <c r="C72">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>73</v>
+      </c>
+      <c r="B73" t="s">
+        <v>938</v>
+      </c>
+      <c r="C73">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>104</v>
+      </c>
+      <c r="C74">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75">
+        <v>75</v>
+      </c>
+      <c r="B75" t="s">
+        <v>63</v>
+      </c>
+      <c r="C75">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>939</v>
+      </c>
+      <c r="C76">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77">
+        <v>77</v>
+      </c>
+      <c r="B77" t="s">
+        <v>492</v>
+      </c>
+      <c r="C77">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>940</v>
+      </c>
+      <c r="C78">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A79">
+        <v>79</v>
+      </c>
+      <c r="B79" t="s">
+        <v>487</v>
+      </c>
+      <c r="C79">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A80">
+        <v>80</v>
+      </c>
+      <c r="B80" t="s">
+        <v>545</v>
+      </c>
+      <c r="C80">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>167</v>
+      </c>
+      <c r="C81">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A82">
+        <v>82</v>
+      </c>
+      <c r="B82" t="s">
+        <v>25</v>
+      </c>
+      <c r="C82">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
+        <v>941</v>
+      </c>
+      <c r="C83">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A84">
+        <v>84</v>
+      </c>
+      <c r="B84" t="s">
+        <v>491</v>
+      </c>
+      <c r="C84">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>490</v>
+      </c>
+      <c r="C85">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A86">
+        <v>86</v>
+      </c>
+      <c r="B86" t="s">
+        <v>942</v>
+      </c>
+      <c r="C86">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
+        <v>373</v>
+      </c>
+      <c r="C87">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A88">
+        <v>86</v>
+      </c>
+      <c r="B88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C88">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A89">
+        <v>89</v>
+      </c>
+      <c r="B89" t="s">
+        <v>287</v>
+      </c>
+      <c r="C89">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>943</v>
+      </c>
+      <c r="C90">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91">
+        <v>91</v>
+      </c>
+      <c r="B91" t="s">
+        <v>944</v>
+      </c>
+      <c r="C91">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A92">
+        <v>92</v>
+      </c>
+      <c r="B92" t="s">
+        <v>945</v>
+      </c>
+      <c r="C92">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A93">
+        <v>93</v>
+      </c>
+      <c r="B93" t="s">
+        <v>122</v>
+      </c>
+      <c r="C93">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A94">
+        <v>94</v>
+      </c>
+      <c r="B94" t="s">
+        <v>946</v>
+      </c>
+      <c r="C94">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>551</v>
+      </c>
+      <c r="C95">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A96">
+        <v>94</v>
+      </c>
+      <c r="B96" t="s">
+        <v>482</v>
+      </c>
+      <c r="C96">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A97">
+        <v>97</v>
+      </c>
+      <c r="B97" t="s">
+        <v>498</v>
+      </c>
+      <c r="C97">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A98">
+        <v>98</v>
+      </c>
+      <c r="B98" t="s">
+        <v>33</v>
+      </c>
+      <c r="C98">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A99">
+        <v>99</v>
+      </c>
+      <c r="B99" t="s">
+        <v>452</v>
+      </c>
+      <c r="C99">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69F7F02A-6B68-0C4F-B03E-012278D8BB25}">
   <dimension ref="A1:C55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -24475,7 +25653,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF51EAFD-3809-A74B-B55F-B64F3DA7F7E5}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -24518,7 +25696,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <dimension ref="A1:C80"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -25412,7 +26590,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <dimension ref="A1:C86"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -26458,7 +27636,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <dimension ref="A1:C90"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -27462,7 +28640,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <dimension ref="A1:C109"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -28675,7 +29853,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
   <dimension ref="A1:C105"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -29844,7 +31022,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
   <dimension ref="A1:C73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -30654,801 +31832,6 @@
       </c>
       <c r="C73" s="2">
         <v>42</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
-  <dimension ref="A1:C71"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="2" width="10.83203125" style="2" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="2">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="C1" s="2">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
-        <v>2</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="2">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="2">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="2">
-        <v>4</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="C4" s="2">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
-        <v>5</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="2">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="2">
-        <v>6</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="C6" s="2">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
-        <v>7</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="2">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="2">
-        <v>8</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C8" s="2">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="2">
-        <v>9</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="C9" s="2">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
-        <v>10</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="C10" s="2">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="2">
-        <v>11</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" s="2">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="2">
-        <v>12</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="C12" s="2">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
-        <v>13</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="2">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="2">
-        <v>14</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C14" s="2">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="2">
-        <v>15</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C15" s="2">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="2">
-        <v>16</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="C16" s="2">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="2">
-        <v>17</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C17" s="2">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="2">
-        <v>18</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="C18" s="2">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="2">
-        <v>19</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C19" s="2">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="2">
-        <v>20</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="C20" s="2">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="2">
-        <v>21</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C21" s="2">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="2">
-        <v>22</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="C22" s="2">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="2">
-        <v>23</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C23" s="2">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="2">
-        <v>24</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="C24" s="2">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="2">
-        <v>25</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="C25" s="2">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="2">
-        <v>26</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C26" s="2">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="2">
-        <v>27</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C27" s="2">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" s="2">
-        <v>28</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="C28" s="2">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" s="2">
-        <v>29</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="C29" s="2">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="2">
-        <v>30</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="C30" s="2">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="2">
-        <v>31</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="C31" s="2">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="2">
-        <v>32</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C32" s="2">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="2">
-        <v>33</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="C33" s="2">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="2">
-        <v>34</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>646</v>
-      </c>
-      <c r="C34" s="2">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="2">
-        <v>35</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C35" s="2">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="2">
-        <v>36</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="C36" s="2">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="2">
-        <v>37</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="C37" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="2">
-        <v>38</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="C38" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="2">
-        <v>39</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C39" s="2">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="2">
-        <v>40</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C40" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="2">
-        <v>41</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>649</v>
-      </c>
-      <c r="C41" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" s="2">
-        <v>42</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="C42" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="2">
-        <v>43</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="C43" s="2">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="2">
-        <v>44</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C44" s="2">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="2">
-        <v>45</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C45" s="2">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46" s="2">
-        <v>46</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="C46" s="2">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" s="2">
-        <v>47</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="C47" s="2">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" s="2">
-        <v>48</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>651</v>
-      </c>
-      <c r="C48" s="2">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" s="2">
-        <v>49</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>382</v>
-      </c>
-      <c r="C49" s="2">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" s="2">
-        <v>50</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>652</v>
-      </c>
-      <c r="C50" s="2">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" s="2">
-        <v>51</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="C51" s="2">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A52" s="2">
-        <v>52</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C52" s="2">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A53" s="2">
-        <v>53</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="C53" s="2">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A54" s="2">
-        <v>54</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="C54" s="2">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="2">
-        <v>55</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>653</v>
-      </c>
-      <c r="C55" s="2">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="2">
-        <v>56</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>654</v>
-      </c>
-      <c r="C56" s="2">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" s="2">
-        <v>57</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C57" s="2">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="2">
-        <v>58</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="C58" s="2">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="2">
-        <v>59</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="C59" s="2">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A60" s="2">
-        <v>60</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>346</v>
-      </c>
-      <c r="C60" s="2">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="2">
-        <v>61</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C61" s="2">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="2">
-        <v>62</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>655</v>
-      </c>
-      <c r="C62" s="2">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="2">
-        <v>63</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>656</v>
-      </c>
-      <c r="C63" s="2">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" s="2">
-        <v>64</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="C64" s="2">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" s="2">
-        <v>65</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>657</v>
-      </c>
-      <c r="C65" s="2">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" s="2">
-        <v>66</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C66" s="2">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A67" s="2">
-        <v>67</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>658</v>
-      </c>
-      <c r="C67" s="2">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" s="2">
-        <v>68</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>643</v>
-      </c>
-      <c r="C68" s="2">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" s="2">
-        <v>69</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="C69" s="2">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" s="2">
-        <v>70</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>626</v>
-      </c>
-      <c r="C70" s="2">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A71" s="2">
-        <v>71</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C71" s="2">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -32397,6 +32780,801 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
+  <dimension ref="A1:C71"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="10.83203125" style="2" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="2">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C1" s="2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="2">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="2">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="2">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C4" s="2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C5" s="2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
+        <v>6</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C6" s="2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="2">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
+        <v>8</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C8" s="2">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="2">
+        <v>9</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C9" s="2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="2">
+        <v>10</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C10" s="2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="2">
+        <v>11</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" s="2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="2">
+        <v>12</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C12" s="2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="2">
+        <v>13</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="2">
+        <v>14</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C14" s="2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="2">
+        <v>15</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="2">
+        <v>16</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C16" s="2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="2">
+        <v>17</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="2">
+        <v>18</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="C18" s="2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="2">
+        <v>19</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C19" s="2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="2">
+        <v>20</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="C20" s="2">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="2">
+        <v>21</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C21" s="2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="2">
+        <v>22</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="C22" s="2">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="2">
+        <v>23</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" s="2">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="2">
+        <v>24</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="C24" s="2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="2">
+        <v>25</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C25" s="2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="2">
+        <v>26</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="2">
+        <v>27</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C27" s="2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="2">
+        <v>28</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C28" s="2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="2">
+        <v>29</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="C29" s="2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="2">
+        <v>30</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C30" s="2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="2">
+        <v>31</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C31" s="2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="2">
+        <v>32</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C32" s="2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="2">
+        <v>33</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C33" s="2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="2">
+        <v>34</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="C34" s="2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="2">
+        <v>35</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C35" s="2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="2">
+        <v>36</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C36" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="2">
+        <v>37</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C37" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="2">
+        <v>38</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="C38" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="2">
+        <v>39</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C39" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="2">
+        <v>40</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C40" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" s="2">
+        <v>41</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="C41" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="2">
+        <v>42</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="C42" s="2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" s="2">
+        <v>43</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C43" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" s="2">
+        <v>44</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C44" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" s="2">
+        <v>45</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C45" s="2">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" s="2">
+        <v>46</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="C46" s="2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="2">
+        <v>47</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="C47" s="2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" s="2">
+        <v>48</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="C48" s="2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" s="2">
+        <v>49</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="C49" s="2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" s="2">
+        <v>50</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="C50" s="2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" s="2">
+        <v>51</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C51" s="2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" s="2">
+        <v>52</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C52" s="2">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" s="2">
+        <v>53</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="C53" s="2">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" s="2">
+        <v>54</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C54" s="2">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" s="2">
+        <v>55</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="C55" s="2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" s="2">
+        <v>56</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="C56" s="2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" s="2">
+        <v>57</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C57" s="2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="2">
+        <v>58</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="C58" s="2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="2">
+        <v>59</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C59" s="2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="2">
+        <v>60</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="C60" s="2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="2">
+        <v>61</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C61" s="2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="2">
+        <v>62</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="C62" s="2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="2">
+        <v>63</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="C63" s="2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="2">
+        <v>64</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="C64" s="2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="2">
+        <v>65</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="C65" s="2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="2">
+        <v>66</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C66" s="2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="2">
+        <v>67</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="C67" s="2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="2">
+        <v>68</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>643</v>
+      </c>
+      <c r="C68" s="2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="2">
+        <v>69</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C69" s="2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="2">
+        <v>70</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="C70" s="2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="2">
+        <v>71</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C71" s="2">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <dimension ref="A1:C94"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -33538,7 +34716,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
   <dimension ref="A1:C78"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -34410,7 +35588,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1D00-000000000000}">
   <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -34996,7 +36174,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
   <dimension ref="A1:C63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -35703,7 +36881,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
   <dimension ref="A1:C102"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -36839,7 +38017,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2000-000000000000}">
   <dimension ref="A1:C87"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -37810,7 +38988,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
   <dimension ref="A1:C93"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -38847,7 +40025,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
   <dimension ref="A1:C91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -39862,7 +41040,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
   <dimension ref="A1:C119"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -41178,922 +42356,6 @@
       </c>
       <c r="C119" s="3">
         <v>18</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
-  <dimension ref="A1:C82"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="2" width="8.83203125" style="3" customWidth="1"/>
-    <col min="3" max="16384" width="8.83203125" style="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="3">
-        <v>1</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="3">
-        <v>2</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="3">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="3">
-        <v>3</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>570</v>
-      </c>
-      <c r="C3" s="3">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="3">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="C4" s="3">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="3">
-        <v>5</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>789</v>
-      </c>
-      <c r="C5" s="3">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="3">
-        <v>6</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>659</v>
-      </c>
-      <c r="C6" s="3">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="3">
-        <v>7</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="3">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>8</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" s="3">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
-        <v>9</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="C9" s="3">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
-        <v>10</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="3">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="3">
-        <v>11</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="3">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
-        <v>12</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="3">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
-        <v>13</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="3">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="3">
-        <v>14</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>573</v>
-      </c>
-      <c r="C14" s="3">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="3">
-        <v>15</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>790</v>
-      </c>
-      <c r="C15" s="3">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="3">
-        <v>16</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C16" s="3">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="3">
-        <v>17</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="C17" s="3">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="3">
-        <v>18</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="C18" s="3">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="3">
-        <v>19</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C19" s="3">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="3">
-        <v>20</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="C20" s="3">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="3">
-        <v>21</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="C21" s="3">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="3">
-        <v>22</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>599</v>
-      </c>
-      <c r="C22" s="3">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="3">
-        <v>23</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C23" s="3">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="3">
-        <v>24</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="C24" s="3">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="3">
-        <v>25</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>632</v>
-      </c>
-      <c r="C25" s="3">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="3">
-        <v>26</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="C26" s="3">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="3">
-        <v>27</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" s="3">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" s="3">
-        <v>28</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="C28" s="3">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" s="3">
-        <v>29</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="C29" s="3">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="3">
-        <v>30</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>614</v>
-      </c>
-      <c r="C30" s="3">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="3">
-        <v>31</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>791</v>
-      </c>
-      <c r="C31" s="3">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="3">
-        <v>32</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="C32" s="3">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="3">
-        <v>33</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C33" s="3">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="3">
-        <v>34</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>361</v>
-      </c>
-      <c r="C34" s="3">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="3">
-        <v>35</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="C35" s="3">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="3">
-        <v>36</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>427</v>
-      </c>
-      <c r="C36" s="3">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="3">
-        <v>37</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="C37" s="3">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="3">
-        <v>38</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="C38" s="3">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="3">
-        <v>39</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="C39" s="3">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="3">
-        <v>40</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>663</v>
-      </c>
-      <c r="C40" s="3">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="3">
-        <v>41</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="C41" s="3">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" s="3">
-        <v>42</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>621</v>
-      </c>
-      <c r="C42" s="3">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="3">
-        <v>43</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="C43" s="3">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="3">
-        <v>44</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>792</v>
-      </c>
-      <c r="C44" s="3">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="3">
-        <v>45</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>644</v>
-      </c>
-      <c r="C45" s="3">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46" s="3">
-        <v>46</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C46" s="3">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" s="3">
-        <v>47</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>619</v>
-      </c>
-      <c r="C47" s="3">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" s="3">
-        <v>48</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="C48" s="3">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" s="3">
-        <v>49</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>403</v>
-      </c>
-      <c r="C49" s="3">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" s="3">
-        <v>50</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C50" s="3">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" s="3">
-        <v>51</v>
-      </c>
-      <c r="B51" s="3" t="s">
-        <v>391</v>
-      </c>
-      <c r="C51" s="3">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A52" s="3">
-        <v>52</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C52" s="3">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A53" s="3">
-        <v>53</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C53" s="3">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A54" s="3">
-        <v>54</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C54" s="3">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="3">
-        <v>55</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C55" s="3">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="3">
-        <v>56</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="C56" s="3">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" s="3">
-        <v>57</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>585</v>
-      </c>
-      <c r="C57" s="3">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="3">
-        <v>58</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C58" s="3">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="3">
-        <v>59</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>507</v>
-      </c>
-      <c r="C59" s="3">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A60" s="3">
-        <v>60</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C60" s="3">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="3">
-        <v>61</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="C61" s="3">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="3">
-        <v>62</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="C62" s="3">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="3">
-        <v>63</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="C63" s="3">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" s="3">
-        <v>64</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="C64" s="3">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" s="3">
-        <v>65</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="C65" s="3">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" s="3">
-        <v>66</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C66" s="3">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A67" s="3">
-        <v>67</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>592</v>
-      </c>
-      <c r="C67" s="3">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" s="3">
-        <v>68</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="C68" s="3">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" s="3">
-        <v>69</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>793</v>
-      </c>
-      <c r="C69" s="3">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" s="3">
-        <v>70</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="C70" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A71" s="3">
-        <v>71</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C71" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" s="3">
-        <v>72</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>638</v>
-      </c>
-      <c r="C72" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A73" s="3">
-        <v>73</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>354</v>
-      </c>
-      <c r="C73" s="3">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A74" s="3">
-        <v>74</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>346</v>
-      </c>
-      <c r="C74" s="3">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A75" s="3">
-        <v>75</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>794</v>
-      </c>
-      <c r="C75" s="3">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A76" s="3">
-        <v>76</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C76" s="3">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A77" s="3">
-        <v>77</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>795</v>
-      </c>
-      <c r="C77" s="3">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A78" s="3">
-        <v>78</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C78" s="3">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A79" s="3">
-        <v>79</v>
-      </c>
-      <c r="B79" s="3" t="s">
-        <v>453</v>
-      </c>
-      <c r="C79" s="3">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A80" s="3">
-        <v>80</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>625</v>
-      </c>
-      <c r="C80" s="3">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A81" s="3">
-        <v>81</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>796</v>
-      </c>
-      <c r="C81" s="3">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A82" s="3">
-        <v>82</v>
-      </c>
-      <c r="B82" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="C82" s="3">
-        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -44316,6 +44578,922 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
+  <dimension ref="A1:C82"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="8.83203125" style="3" customWidth="1"/>
+    <col min="3" max="16384" width="8.83203125" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="3">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="3">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="3">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C3" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C4" s="3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="3">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>789</v>
+      </c>
+      <c r="C5" s="3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="3">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>659</v>
+      </c>
+      <c r="C6" s="3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>7</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>8</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C9" s="3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="3">
+        <v>10</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
+        <v>11</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="3">
+        <v>12</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="3">
+        <v>13</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="3">
+        <v>14</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="C14" s="3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="3">
+        <v>15</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>790</v>
+      </c>
+      <c r="C15" s="3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="3">
+        <v>16</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C16" s="3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="3">
+        <v>17</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C17" s="3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="3">
+        <v>18</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C18" s="3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="3">
+        <v>19</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C19" s="3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="3">
+        <v>20</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="C20" s="3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="3">
+        <v>21</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C21" s="3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="3">
+        <v>22</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>599</v>
+      </c>
+      <c r="C22" s="3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="3">
+        <v>23</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="3">
+        <v>24</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" s="3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>25</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="C25" s="3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="3">
+        <v>26</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="C26" s="3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="3">
+        <v>27</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" s="3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="3">
+        <v>28</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="C28" s="3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="3">
+        <v>29</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="C29" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="3">
+        <v>30</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="C30" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="3">
+        <v>31</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>791</v>
+      </c>
+      <c r="C31" s="3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="3">
+        <v>32</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C32" s="3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="3">
+        <v>33</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C33" s="3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="3">
+        <v>34</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="C34" s="3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="3">
+        <v>35</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="C35" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="3">
+        <v>36</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="C36" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="3">
+        <v>37</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="C37" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="3">
+        <v>38</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C38" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="3">
+        <v>39</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="C39" s="3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="3">
+        <v>40</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>663</v>
+      </c>
+      <c r="C40" s="3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" s="3">
+        <v>41</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C41" s="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="3">
+        <v>42</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>621</v>
+      </c>
+      <c r="C42" s="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" s="3">
+        <v>43</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="C43" s="3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" s="3">
+        <v>44</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="C44" s="3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" s="3">
+        <v>45</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>644</v>
+      </c>
+      <c r="C45" s="3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" s="3">
+        <v>46</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C46" s="3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <v>47</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>619</v>
+      </c>
+      <c r="C47" s="3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" s="3">
+        <v>48</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="C48" s="3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" s="3">
+        <v>49</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="C49" s="3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" s="3">
+        <v>50</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C50" s="3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" s="3">
+        <v>51</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="C51" s="3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" s="3">
+        <v>52</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C52" s="3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" s="3">
+        <v>53</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C53" s="3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" s="3">
+        <v>54</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C54" s="3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" s="3">
+        <v>55</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C55" s="3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" s="3">
+        <v>56</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C56" s="3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" s="3">
+        <v>57</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="C57" s="3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="3">
+        <v>58</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C58" s="3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="3">
+        <v>59</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="C59" s="3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="3">
+        <v>60</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C60" s="3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="3">
+        <v>61</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="C61" s="3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="3">
+        <v>62</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C62" s="3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="3">
+        <v>63</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="C63" s="3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="3">
+        <v>64</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C64" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="3">
+        <v>65</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="C65" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="3">
+        <v>66</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C66" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="3">
+        <v>67</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="C67" s="3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="3">
+        <v>68</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="C68" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="3">
+        <v>69</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>793</v>
+      </c>
+      <c r="C69" s="3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="3">
+        <v>70</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C70" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="3">
+        <v>71</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C71" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="3">
+        <v>72</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>638</v>
+      </c>
+      <c r="C72" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="3">
+        <v>73</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C73" s="3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74" s="3">
+        <v>74</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="C74" s="3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75" s="3">
+        <v>75</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>794</v>
+      </c>
+      <c r="C75" s="3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76" s="3">
+        <v>76</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C76" s="3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77" s="3">
+        <v>77</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>795</v>
+      </c>
+      <c r="C77" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A78" s="3">
+        <v>78</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C78" s="3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A79" s="3">
+        <v>79</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="C79" s="3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A80" s="3">
+        <v>80</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="C80" s="3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A81" s="3">
+        <v>81</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="C81" s="3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A82" s="3">
+        <v>82</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C82" s="3">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
   <dimension ref="A1:C173"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -46232,7 +47410,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <dimension ref="A1:C200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -48446,7 +49624,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
   <dimension ref="A1:C118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -49758,7 +50936,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2800-000000000000}">
   <dimension ref="A1:C79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
feat: add cro open 2016
</commit_message>
<xml_diff>
--- a/rank.xlsx
+++ b/rank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neven/Documents/github-repos/croatian-quiz-scores/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04899E9C-A298-BC4E-A854-15F0F82684FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD6238A9-DD6A-5C48-B5BD-42E617C6EBF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19220" firstSheet="16" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6840" yWindow="600" windowWidth="31560" windowHeight="19220" firstSheet="16" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SOVA 2017" sheetId="1" r:id="rId1"/>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4135" uniqueCount="947">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4207" uniqueCount="956">
   <si>
     <t>Krešimir Štimac</t>
   </si>
@@ -2916,6 +2916,33 @@
   </si>
   <si>
     <t>Filip Špoljarić</t>
+  </si>
+  <si>
+    <t>Josip Kelava</t>
+  </si>
+  <si>
+    <t>Ivan-Filip Maček</t>
+  </si>
+  <si>
+    <t>Igor Milković</t>
+  </si>
+  <si>
+    <t>Branimir Magaš</t>
+  </si>
+  <si>
+    <t>Antonela Gajdek</t>
+  </si>
+  <si>
+    <t>Josip Luša</t>
+  </si>
+  <si>
+    <t>Hrvoje Marin</t>
+  </si>
+  <si>
+    <t>Stephanie-Ruth Hamp</t>
+  </si>
+  <si>
+    <t>Hrvoje Milošević</t>
   </si>
 </sst>
 </file>
@@ -25655,7 +25682,7 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF51EAFD-3809-A74B-B55F-B64F3DA7F7E5}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -25666,7 +25693,7 @@
         <v>2</v>
       </c>
       <c r="C1">
-        <v>112</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -25677,7 +25704,7 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>108</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -25688,7 +25715,799 @@
         <v>0</v>
       </c>
       <c r="C3">
-        <v>105</v>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>570</v>
+      </c>
+      <c r="C4">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>225</v>
+      </c>
+      <c r="C10">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>133</v>
+      </c>
+      <c r="C11">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>129</v>
+      </c>
+      <c r="C16">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>17</v>
+      </c>
+      <c r="B17" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>18</v>
+      </c>
+      <c r="B18" t="s">
+        <v>131</v>
+      </c>
+      <c r="C18">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>19</v>
+      </c>
+      <c r="B19" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>20</v>
+      </c>
+      <c r="B20" t="s">
+        <v>259</v>
+      </c>
+      <c r="C20">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>21</v>
+      </c>
+      <c r="B21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>22</v>
+      </c>
+      <c r="B22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>23</v>
+      </c>
+      <c r="B23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>24</v>
+      </c>
+      <c r="B24" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>27</v>
+      </c>
+      <c r="B27" t="s">
+        <v>921</v>
+      </c>
+      <c r="C27">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>28</v>
+      </c>
+      <c r="B28" t="s">
+        <v>684</v>
+      </c>
+      <c r="C28">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>29</v>
+      </c>
+      <c r="B29" t="s">
+        <v>165</v>
+      </c>
+      <c r="C29">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>30</v>
+      </c>
+      <c r="B30" t="s">
+        <v>947</v>
+      </c>
+      <c r="C30">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>31</v>
+      </c>
+      <c r="B31" t="s">
+        <v>13</v>
+      </c>
+      <c r="C31">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>32</v>
+      </c>
+      <c r="B32" t="s">
+        <v>948</v>
+      </c>
+      <c r="C32">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>33</v>
+      </c>
+      <c r="B33" t="s">
+        <v>206</v>
+      </c>
+      <c r="C33">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>881</v>
+      </c>
+      <c r="C34">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>35</v>
+      </c>
+      <c r="B35" t="s">
+        <v>901</v>
+      </c>
+      <c r="C35">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>36</v>
+      </c>
+      <c r="B36" t="s">
+        <v>63</v>
+      </c>
+      <c r="C36">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>37</v>
+      </c>
+      <c r="B37" t="s">
+        <v>400</v>
+      </c>
+      <c r="C37">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>949</v>
+      </c>
+      <c r="C38">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>39</v>
+      </c>
+      <c r="B39" t="s">
+        <v>571</v>
+      </c>
+      <c r="C39">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>40</v>
+      </c>
+      <c r="B40" t="s">
+        <v>573</v>
+      </c>
+      <c r="C40">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>715</v>
+      </c>
+      <c r="C41">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>42</v>
+      </c>
+      <c r="B42" t="s">
+        <v>719</v>
+      </c>
+      <c r="C42">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>58</v>
+      </c>
+      <c r="C43">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>44</v>
+      </c>
+      <c r="B44" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>45</v>
+      </c>
+      <c r="B45" t="s">
+        <v>23</v>
+      </c>
+      <c r="C45">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>54</v>
+      </c>
+      <c r="C46">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>47</v>
+      </c>
+      <c r="B47" t="s">
+        <v>886</v>
+      </c>
+      <c r="C47">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>22</v>
+      </c>
+      <c r="C48">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>49</v>
+      </c>
+      <c r="B49" t="s">
+        <v>950</v>
+      </c>
+      <c r="C49">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>50</v>
+      </c>
+      <c r="B50" t="s">
+        <v>951</v>
+      </c>
+      <c r="C50">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>51</v>
+      </c>
+      <c r="B51" t="s">
+        <v>706</v>
+      </c>
+      <c r="C51">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>52</v>
+      </c>
+      <c r="B52" t="s">
+        <v>26</v>
+      </c>
+      <c r="C52">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>722</v>
+      </c>
+      <c r="C53">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>52</v>
+      </c>
+      <c r="B54" t="s">
+        <v>590</v>
+      </c>
+      <c r="C54">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>55</v>
+      </c>
+      <c r="B55" t="s">
+        <v>66</v>
+      </c>
+      <c r="C55">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>56</v>
+      </c>
+      <c r="B56" t="s">
+        <v>28</v>
+      </c>
+      <c r="C56">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>952</v>
+      </c>
+      <c r="C57">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>58</v>
+      </c>
+      <c r="B58" t="s">
+        <v>86</v>
+      </c>
+      <c r="C58">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>59</v>
+      </c>
+      <c r="B59" t="s">
+        <v>242</v>
+      </c>
+      <c r="C59">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60">
+        <v>60</v>
+      </c>
+      <c r="B60" t="s">
+        <v>25</v>
+      </c>
+      <c r="C60">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61">
+        <v>61</v>
+      </c>
+      <c r="B61" t="s">
+        <v>953</v>
+      </c>
+      <c r="C61">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62">
+        <v>62</v>
+      </c>
+      <c r="B62" t="s">
+        <v>954</v>
+      </c>
+      <c r="C62">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63">
+        <v>63</v>
+      </c>
+      <c r="B63" t="s">
+        <v>74</v>
+      </c>
+      <c r="C63">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>82</v>
+      </c>
+      <c r="C64">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>65</v>
+      </c>
+      <c r="B65" t="s">
+        <v>31</v>
+      </c>
+      <c r="C65">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>38</v>
+      </c>
+      <c r="C66">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>67</v>
+      </c>
+      <c r="B67" t="s">
+        <v>729</v>
+      </c>
+      <c r="C67">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>68</v>
+      </c>
+      <c r="B68" t="s">
+        <v>36</v>
+      </c>
+      <c r="C68">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>69</v>
+      </c>
+      <c r="B69" t="s">
+        <v>30</v>
+      </c>
+      <c r="C69">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>70</v>
+      </c>
+      <c r="B70" t="s">
+        <v>897</v>
+      </c>
+      <c r="C70">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>71</v>
+      </c>
+      <c r="B71" t="s">
+        <v>33</v>
+      </c>
+      <c r="C71">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>32</v>
+      </c>
+      <c r="C72">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>71</v>
+      </c>
+      <c r="B73" t="s">
+        <v>955</v>
+      </c>
+      <c r="C73">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>74</v>
+      </c>
+      <c r="B74" t="s">
+        <v>41</v>
+      </c>
+      <c r="C74">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75">
+        <v>75</v>
+      </c>
+      <c r="B75" t="s">
+        <v>119</v>
+      </c>
+      <c r="C75">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add wqc 2026
</commit_message>
<xml_diff>
--- a/rank.xlsx
+++ b/rank.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neven/Documents/github-repos/croatian-quiz-scores/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A50134A8-B6A7-C34E-816E-CA538D6E7AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8356AC77-F1C6-D24B-8C3E-45D3D36413E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15620" firstSheet="23" activeTab="30" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15620" firstSheet="30" activeTab="35" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SOVA 2017" sheetId="1" r:id="rId1"/>
@@ -48,15 +48,16 @@
     <sheet name="WQC 2014" sheetId="30" r:id="rId33"/>
     <sheet name="WQC 2015" sheetId="31" r:id="rId34"/>
     <sheet name="WQC 2025" sheetId="32" r:id="rId35"/>
-    <sheet name="WQC 2024" sheetId="33" r:id="rId36"/>
-    <sheet name="WQC 2023" sheetId="34" r:id="rId37"/>
-    <sheet name="WQC 2022" sheetId="35" r:id="rId38"/>
-    <sheet name="WQC 2021" sheetId="36" r:id="rId39"/>
-    <sheet name="WQC 2020" sheetId="37" r:id="rId40"/>
-    <sheet name="WQC 2019" sheetId="38" r:id="rId41"/>
-    <sheet name="WQC 2018" sheetId="39" r:id="rId42"/>
-    <sheet name="WQC 2017" sheetId="40" r:id="rId43"/>
-    <sheet name="WQC 2016" sheetId="41" r:id="rId44"/>
+    <sheet name="WQC 2026" sheetId="47" r:id="rId36"/>
+    <sheet name="WQC 2024" sheetId="33" r:id="rId37"/>
+    <sheet name="WQC 2023" sheetId="34" r:id="rId38"/>
+    <sheet name="WQC 2022" sheetId="35" r:id="rId39"/>
+    <sheet name="WQC 2021" sheetId="36" r:id="rId40"/>
+    <sheet name="WQC 2020" sheetId="37" r:id="rId41"/>
+    <sheet name="WQC 2019" sheetId="38" r:id="rId42"/>
+    <sheet name="WQC 2018" sheetId="39" r:id="rId43"/>
+    <sheet name="WQC 2017" sheetId="40" r:id="rId44"/>
+    <sheet name="WQC 2016" sheetId="41" r:id="rId45"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -75,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4207" uniqueCount="955">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4313" uniqueCount="966">
   <si>
     <t>Krešimir Štimac</t>
   </si>
@@ -2940,6 +2941,39 @@
   </si>
   <si>
     <t>Hrvoje Milošević</t>
+  </si>
+  <si>
+    <t>Mihovil Parčina</t>
+  </si>
+  <si>
+    <t>Davor Prpić</t>
+  </si>
+  <si>
+    <t>Marko Kovačić</t>
+  </si>
+  <si>
+    <t>Marko Pongrac</t>
+  </si>
+  <si>
+    <t>David Krajinović</t>
+  </si>
+  <si>
+    <t>Antonio Rabuzin</t>
+  </si>
+  <si>
+    <t>Ivan Strizić</t>
+  </si>
+  <si>
+    <t>Ivan Kaučić</t>
+  </si>
+  <si>
+    <t>Hrvoje Ðurak</t>
+  </si>
+  <si>
+    <t>Dejan Zatezalo</t>
+  </si>
+  <si>
+    <t>Sergije Michieli</t>
   </si>
 </sst>
 </file>
@@ -38842,11 +38876,1191 @@
 </file>
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48222230-6720-4C49-9F89-FD6BE3B5DBF5}">
+  <dimension ref="A1:C106"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="20.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C2">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>158</v>
+      </c>
+      <c r="C6">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>342</v>
+      </c>
+      <c r="C8">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>503</v>
+      </c>
+      <c r="C9">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>393</v>
+      </c>
+      <c r="C11">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>260</v>
+      </c>
+      <c r="C12">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>13</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>570</v>
+      </c>
+      <c r="C14">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>15</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>140</v>
+      </c>
+      <c r="C16">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>17</v>
+      </c>
+      <c r="B17" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>18</v>
+      </c>
+      <c r="B18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>19</v>
+      </c>
+      <c r="B19" t="s">
+        <v>659</v>
+      </c>
+      <c r="C19">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>20</v>
+      </c>
+      <c r="B20" t="s">
+        <v>955</v>
+      </c>
+      <c r="C20">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>21</v>
+      </c>
+      <c r="B21" t="s">
+        <v>391</v>
+      </c>
+      <c r="C21">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>22</v>
+      </c>
+      <c r="B22" t="s">
+        <v>382</v>
+      </c>
+      <c r="C22">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>23</v>
+      </c>
+      <c r="B23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>24</v>
+      </c>
+      <c r="B24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>25</v>
+      </c>
+      <c r="B25" t="s">
+        <v>129</v>
+      </c>
+      <c r="C25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>26</v>
+      </c>
+      <c r="B26" t="s">
+        <v>506</v>
+      </c>
+      <c r="C26">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>27</v>
+      </c>
+      <c r="B27" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>28</v>
+      </c>
+      <c r="B28" t="s">
+        <v>518</v>
+      </c>
+      <c r="C28">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>29</v>
+      </c>
+      <c r="B29" t="s">
+        <v>435</v>
+      </c>
+      <c r="C29">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>30</v>
+      </c>
+      <c r="B30" t="s">
+        <v>189</v>
+      </c>
+      <c r="C30">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>31</v>
+      </c>
+      <c r="B31" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>32</v>
+      </c>
+      <c r="B32" t="s">
+        <v>956</v>
+      </c>
+      <c r="C32">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>33</v>
+      </c>
+      <c r="B33" t="s">
+        <v>507</v>
+      </c>
+      <c r="C33">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>34</v>
+      </c>
+      <c r="B34" t="s">
+        <v>673</v>
+      </c>
+      <c r="C34">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>35</v>
+      </c>
+      <c r="B35" t="s">
+        <v>280</v>
+      </c>
+      <c r="C35">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>36</v>
+      </c>
+      <c r="B36" t="s">
+        <v>131</v>
+      </c>
+      <c r="C36">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>37</v>
+      </c>
+      <c r="B37" t="s">
+        <v>427</v>
+      </c>
+      <c r="C37">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>38</v>
+      </c>
+      <c r="B38" t="s">
+        <v>191</v>
+      </c>
+      <c r="C38">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>39</v>
+      </c>
+      <c r="B39" t="s">
+        <v>441</v>
+      </c>
+      <c r="C39">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>40</v>
+      </c>
+      <c r="B40" t="s">
+        <v>353</v>
+      </c>
+      <c r="C40">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>41</v>
+      </c>
+      <c r="B41" t="s">
+        <v>514</v>
+      </c>
+      <c r="C41">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>42</v>
+      </c>
+      <c r="B42" t="s">
+        <v>46</v>
+      </c>
+      <c r="C42">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>43</v>
+      </c>
+      <c r="B43" t="s">
+        <v>75</v>
+      </c>
+      <c r="C43">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>44</v>
+      </c>
+      <c r="B44" t="s">
+        <v>59</v>
+      </c>
+      <c r="C44">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>45</v>
+      </c>
+      <c r="B45" t="s">
+        <v>489</v>
+      </c>
+      <c r="C45">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>46</v>
+      </c>
+      <c r="B46" t="s">
+        <v>573</v>
+      </c>
+      <c r="C46">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>47</v>
+      </c>
+      <c r="B47" t="s">
+        <v>572</v>
+      </c>
+      <c r="C47">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>48</v>
+      </c>
+      <c r="B48" t="s">
+        <v>780</v>
+      </c>
+      <c r="C48">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>49</v>
+      </c>
+      <c r="B49" t="s">
+        <v>43</v>
+      </c>
+      <c r="C49">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>50</v>
+      </c>
+      <c r="B50" t="s">
+        <v>558</v>
+      </c>
+      <c r="C50">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>51</v>
+      </c>
+      <c r="B51" t="s">
+        <v>399</v>
+      </c>
+      <c r="C51">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>52</v>
+      </c>
+      <c r="B52" t="s">
+        <v>154</v>
+      </c>
+      <c r="C52">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>53</v>
+      </c>
+      <c r="B53" t="s">
+        <v>279</v>
+      </c>
+      <c r="C53">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>54</v>
+      </c>
+      <c r="B54" t="s">
+        <v>14</v>
+      </c>
+      <c r="C54">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>55</v>
+      </c>
+      <c r="B55" t="s">
+        <v>398</v>
+      </c>
+      <c r="C55">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>56</v>
+      </c>
+      <c r="B56" t="s">
+        <v>362</v>
+      </c>
+      <c r="C56">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>57</v>
+      </c>
+      <c r="B57" t="s">
+        <v>615</v>
+      </c>
+      <c r="C57">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>58</v>
+      </c>
+      <c r="B58" t="s">
+        <v>934</v>
+      </c>
+      <c r="C58">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>59</v>
+      </c>
+      <c r="B59" t="s">
+        <v>957</v>
+      </c>
+      <c r="C59">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60">
+        <v>60</v>
+      </c>
+      <c r="B60" t="s">
+        <v>480</v>
+      </c>
+      <c r="C60">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61">
+        <v>61</v>
+      </c>
+      <c r="B61" t="s">
+        <v>958</v>
+      </c>
+      <c r="C61">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62">
+        <v>62</v>
+      </c>
+      <c r="B62" t="s">
+        <v>104</v>
+      </c>
+      <c r="C62">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63">
+        <v>63</v>
+      </c>
+      <c r="B63" t="s">
+        <v>446</v>
+      </c>
+      <c r="C63">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64">
+        <v>64</v>
+      </c>
+      <c r="B64" t="s">
+        <v>745</v>
+      </c>
+      <c r="C64">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>65</v>
+      </c>
+      <c r="B65" t="s">
+        <v>433</v>
+      </c>
+      <c r="C65">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>66</v>
+      </c>
+      <c r="B66" t="s">
+        <v>234</v>
+      </c>
+      <c r="C66">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>67</v>
+      </c>
+      <c r="B67" t="s">
+        <v>536</v>
+      </c>
+      <c r="C67">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>68</v>
+      </c>
+      <c r="B68" t="s">
+        <v>198</v>
+      </c>
+      <c r="C68">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>69</v>
+      </c>
+      <c r="B69" t="s">
+        <v>760</v>
+      </c>
+      <c r="C69">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>70</v>
+      </c>
+      <c r="B70" t="s">
+        <v>567</v>
+      </c>
+      <c r="C70">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>71</v>
+      </c>
+      <c r="B71" t="s">
+        <v>313</v>
+      </c>
+      <c r="C71">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>72</v>
+      </c>
+      <c r="B72" t="s">
+        <v>63</v>
+      </c>
+      <c r="C72">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>73</v>
+      </c>
+      <c r="B73" t="s">
+        <v>935</v>
+      </c>
+      <c r="C73">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>74</v>
+      </c>
+      <c r="B74" t="s">
+        <v>188</v>
+      </c>
+      <c r="C74">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75">
+        <v>75</v>
+      </c>
+      <c r="B75" t="s">
+        <v>675</v>
+      </c>
+      <c r="C75">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76">
+        <v>76</v>
+      </c>
+      <c r="B76" t="s">
+        <v>678</v>
+      </c>
+      <c r="C76">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77">
+        <v>77</v>
+      </c>
+      <c r="B77" t="s">
+        <v>453</v>
+      </c>
+      <c r="C77">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A78">
+        <v>78</v>
+      </c>
+      <c r="B78" t="s">
+        <v>959</v>
+      </c>
+      <c r="C78">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A79">
+        <v>79</v>
+      </c>
+      <c r="B79" t="s">
+        <v>714</v>
+      </c>
+      <c r="C79">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A80">
+        <v>80</v>
+      </c>
+      <c r="B80" t="s">
+        <v>650</v>
+      </c>
+      <c r="C80">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A81">
+        <v>81</v>
+      </c>
+      <c r="B81" t="s">
+        <v>664</v>
+      </c>
+      <c r="C81">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A82">
+        <v>82</v>
+      </c>
+      <c r="B82" t="s">
+        <v>747</v>
+      </c>
+      <c r="C82">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A83">
+        <v>83</v>
+      </c>
+      <c r="B83" t="s">
+        <v>551</v>
+      </c>
+      <c r="C83">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A84">
+        <v>84</v>
+      </c>
+      <c r="B84" t="s">
+        <v>477</v>
+      </c>
+      <c r="C84">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A85">
+        <v>85</v>
+      </c>
+      <c r="B85" t="s">
+        <v>960</v>
+      </c>
+      <c r="C85">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A86">
+        <v>86</v>
+      </c>
+      <c r="B86" t="s">
+        <v>666</v>
+      </c>
+      <c r="C86">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A87">
+        <v>87</v>
+      </c>
+      <c r="B87" t="s">
+        <v>562</v>
+      </c>
+      <c r="C87">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A88">
+        <v>88</v>
+      </c>
+      <c r="B88" t="s">
+        <v>652</v>
+      </c>
+      <c r="C88">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A89">
+        <v>89</v>
+      </c>
+      <c r="B89" t="s">
+        <v>945</v>
+      </c>
+      <c r="C89">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90">
+        <v>90</v>
+      </c>
+      <c r="B90" t="s">
+        <v>529</v>
+      </c>
+      <c r="C90">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91">
+        <v>91</v>
+      </c>
+      <c r="B91" t="s">
+        <v>642</v>
+      </c>
+      <c r="C91">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A92">
+        <v>92</v>
+      </c>
+      <c r="B92" t="s">
+        <v>961</v>
+      </c>
+      <c r="C92">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A93">
+        <v>93</v>
+      </c>
+      <c r="B93" t="s">
+        <v>454</v>
+      </c>
+      <c r="C93">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A94">
+        <v>94</v>
+      </c>
+      <c r="B94" t="s">
+        <v>479</v>
+      </c>
+      <c r="C94">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A95">
+        <v>95</v>
+      </c>
+      <c r="B95" t="s">
+        <v>464</v>
+      </c>
+      <c r="C95">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A96">
+        <v>96</v>
+      </c>
+      <c r="B96" t="s">
+        <v>593</v>
+      </c>
+      <c r="C96">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A97">
+        <v>97</v>
+      </c>
+      <c r="B97" t="s">
+        <v>335</v>
+      </c>
+      <c r="C97">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A98">
+        <v>98</v>
+      </c>
+      <c r="B98" t="s">
+        <v>962</v>
+      </c>
+      <c r="C98">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A99">
+        <v>99</v>
+      </c>
+      <c r="B99" t="s">
+        <v>963</v>
+      </c>
+      <c r="C99">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A100">
+        <v>100</v>
+      </c>
+      <c r="B100" t="s">
+        <v>28</v>
+      </c>
+      <c r="C100">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A101">
+        <v>101</v>
+      </c>
+      <c r="B101" t="s">
+        <v>539</v>
+      </c>
+      <c r="C101">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A102">
+        <v>102</v>
+      </c>
+      <c r="B102" t="s">
+        <v>569</v>
+      </c>
+      <c r="C102">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A103">
+        <v>103</v>
+      </c>
+      <c r="B103" t="s">
+        <v>249</v>
+      </c>
+      <c r="C103">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A104">
+        <v>104</v>
+      </c>
+      <c r="B104" t="s">
+        <v>964</v>
+      </c>
+      <c r="C104">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A105">
+        <v>105</v>
+      </c>
+      <c r="B105" t="s">
+        <v>830</v>
+      </c>
+      <c r="C105">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A106">
+        <v>106</v>
+      </c>
+      <c r="B106" t="s">
+        <v>965</v>
+      </c>
+      <c r="C106">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2000-000000000000}">
   <dimension ref="A1:C87"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="8.83203125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20.1640625" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="16384" width="8.83203125" style="3"/>
   </cols>
   <sheetData>
@@ -39812,7 +41026,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
   <dimension ref="A1:C93"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -40849,7 +42063,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
   <dimension ref="A1:C91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -41857,1329 +43071,6 @@
       </c>
       <c r="C91" s="3">
         <v>33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
-  <dimension ref="A1:C119"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="2" width="8.83203125" style="3" customWidth="1"/>
-    <col min="3" max="16384" width="8.83203125" style="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="3">
-        <v>1</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="3">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="3">
-        <v>2</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="3">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="3">
-        <v>3</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="3">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="3">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>570</v>
-      </c>
-      <c r="C4" s="3">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="3">
-        <v>5</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="C5" s="3">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="3">
-        <v>6</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="C6" s="3">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="3">
-        <v>7</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="3">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>8</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
-        <v>9</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C9" s="3">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
-        <v>10</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="3">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="3">
-        <v>11</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C11" s="3">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
-        <v>12</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C12" s="3">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
-        <v>13</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C13" s="3">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="3">
-        <v>14</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="3">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="3">
-        <v>15</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="3">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="3">
-        <v>16</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C16" s="3">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="3">
-        <v>17</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" s="3">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="3">
-        <v>18</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="C18" s="3">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="3">
-        <v>19</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="C19" s="3">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="3">
-        <v>20</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="C20" s="3">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="3">
-        <v>21</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C21" s="3">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="3">
-        <v>22</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="C22" s="3">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="3">
-        <v>23</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C23" s="3">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="3">
-        <v>24</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C24" s="3">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="3">
-        <v>25</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C25" s="3">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="3">
-        <v>26</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C26" s="3">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="3">
-        <v>27</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="C27" s="3">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" s="3">
-        <v>28</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C28" s="3">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" s="3">
-        <v>29</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C29" s="3">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="3">
-        <v>30</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="C30" s="3">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="3">
-        <v>31</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="C31" s="3">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="3">
-        <v>32</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C32" s="3">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="3">
-        <v>33</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C33" s="3">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="3">
-        <v>34</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C34" s="3">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="3">
-        <v>35</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C35" s="3">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="3">
-        <v>36</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C36" s="3">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="3">
-        <v>37</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="C37" s="3">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="3">
-        <v>38</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C38" s="3">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="3">
-        <v>39</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="C39" s="3">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="3">
-        <v>40</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C40" s="3">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="3">
-        <v>41</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="C41" s="3">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" s="3">
-        <v>42</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="C42" s="3">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="3">
-        <v>43</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>681</v>
-      </c>
-      <c r="C43" s="3">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="3">
-        <v>44</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="C44" s="3">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="3">
-        <v>45</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="C45" s="3">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46" s="3">
-        <v>46</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="C46" s="3">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" s="3">
-        <v>47</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>573</v>
-      </c>
-      <c r="C47" s="3">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" s="3">
-        <v>48</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>614</v>
-      </c>
-      <c r="C48" s="3">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" s="3">
-        <v>49</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="C49" s="3">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" s="3">
-        <v>50</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="C50" s="3">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" s="3">
-        <v>51</v>
-      </c>
-      <c r="B51" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C51" s="3">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A52" s="3">
-        <v>52</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="C52" s="3">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A53" s="3">
-        <v>53</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="C53" s="3">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A54" s="3">
-        <v>54</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>313</v>
-      </c>
-      <c r="C54" s="3">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="3">
-        <v>55</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C55" s="3">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="3">
-        <v>56</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>631</v>
-      </c>
-      <c r="C56" s="3">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" s="3">
-        <v>57</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>354</v>
-      </c>
-      <c r="C57" s="3">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="3">
-        <v>58</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="C58" s="3">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="3">
-        <v>59</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C59" s="3">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A60" s="3">
-        <v>60</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C60" s="3">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="3">
-        <v>61</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C61" s="3">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="3">
-        <v>62</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="C62" s="3">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="3">
-        <v>63</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="C63" s="3">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" s="3">
-        <v>64</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C64" s="3">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" s="3">
-        <v>65</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="C65" s="3">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" s="3">
-        <v>66</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>780</v>
-      </c>
-      <c r="C66" s="3">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A67" s="3">
-        <v>67</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="C67" s="3">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" s="3">
-        <v>68</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C68" s="3">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" s="3">
-        <v>69</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="C69" s="3">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" s="3">
-        <v>70</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C70" s="3">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A71" s="3">
-        <v>71</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C71" s="3">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" s="3">
-        <v>72</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="C72" s="3">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A73" s="3">
-        <v>73</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="C73" s="3">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A74" s="3">
-        <v>74</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C74" s="3">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A75" s="3">
-        <v>75</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="C75" s="3">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A76" s="3">
-        <v>76</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>714</v>
-      </c>
-      <c r="C76" s="3">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A77" s="3">
-        <v>77</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>782</v>
-      </c>
-      <c r="C77" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A78" s="3">
-        <v>78</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>632</v>
-      </c>
-      <c r="C78" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A79" s="3">
-        <v>79</v>
-      </c>
-      <c r="B79" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="C79" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A80" s="3">
-        <v>80</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="C80" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A81" s="3">
-        <v>81</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="C81" s="3">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A82" s="3">
-        <v>82</v>
-      </c>
-      <c r="B82" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="C82" s="3">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A83" s="3">
-        <v>83</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>744</v>
-      </c>
-      <c r="C83" s="3">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A84" s="3">
-        <v>84</v>
-      </c>
-      <c r="B84" s="3" t="s">
-        <v>621</v>
-      </c>
-      <c r="C84" s="3">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A85" s="3">
-        <v>85</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>321</v>
-      </c>
-      <c r="C85" s="3">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A86" s="3">
-        <v>86</v>
-      </c>
-      <c r="B86" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="C86" s="3">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A87" s="3">
-        <v>87</v>
-      </c>
-      <c r="B87" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="C87" s="3">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A88" s="3">
-        <v>88</v>
-      </c>
-      <c r="B88" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="C88" s="3">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A89" s="3">
-        <v>89</v>
-      </c>
-      <c r="B89" s="3" t="s">
-        <v>644</v>
-      </c>
-      <c r="C89" s="3">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A90" s="3">
-        <v>90</v>
-      </c>
-      <c r="B90" s="3" t="s">
-        <v>705</v>
-      </c>
-      <c r="C90" s="3">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A91" s="3">
-        <v>91</v>
-      </c>
-      <c r="B91" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C91" s="3">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A92" s="3">
-        <v>92</v>
-      </c>
-      <c r="B92" s="3" t="s">
-        <v>641</v>
-      </c>
-      <c r="C92" s="3">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A93" s="3">
-        <v>93</v>
-      </c>
-      <c r="B93" s="3" t="s">
-        <v>600</v>
-      </c>
-      <c r="C93" s="3">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A94" s="3">
-        <v>94</v>
-      </c>
-      <c r="B94" s="3" t="s">
-        <v>783</v>
-      </c>
-      <c r="C94" s="3">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A95" s="3">
-        <v>95</v>
-      </c>
-      <c r="B95" s="3" t="s">
-        <v>593</v>
-      </c>
-      <c r="C95" s="3">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A96" s="3">
-        <v>96</v>
-      </c>
-      <c r="B96" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C96" s="3">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A97" s="3">
-        <v>97</v>
-      </c>
-      <c r="B97" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="C97" s="3">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A98" s="3">
-        <v>98</v>
-      </c>
-      <c r="B98" s="3" t="s">
-        <v>639</v>
-      </c>
-      <c r="C98" s="3">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A99" s="3">
-        <v>99</v>
-      </c>
-      <c r="B99" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C99" s="3">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A100" s="3">
-        <v>100</v>
-      </c>
-      <c r="B100" s="3" t="s">
-        <v>778</v>
-      </c>
-      <c r="C100" s="3">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A101" s="3">
-        <v>101</v>
-      </c>
-      <c r="B101" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C101" s="3">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A102" s="3">
-        <v>102</v>
-      </c>
-      <c r="B102" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C102" s="3">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A103" s="3">
-        <v>103</v>
-      </c>
-      <c r="B103" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C103" s="3">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A104" s="3">
-        <v>104</v>
-      </c>
-      <c r="B104" s="3" t="s">
-        <v>607</v>
-      </c>
-      <c r="C104" s="3">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A105" s="3">
-        <v>105</v>
-      </c>
-      <c r="B105" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C105" s="3">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A106" s="3">
-        <v>106</v>
-      </c>
-      <c r="B106" s="3" t="s">
-        <v>361</v>
-      </c>
-      <c r="C106" s="3">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A107" s="3">
-        <v>107</v>
-      </c>
-      <c r="B107" s="3" t="s">
-        <v>453</v>
-      </c>
-      <c r="C107" s="3">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A108" s="3">
-        <v>108</v>
-      </c>
-      <c r="B108" s="3" t="s">
-        <v>608</v>
-      </c>
-      <c r="C108" s="3">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A109" s="3">
-        <v>109</v>
-      </c>
-      <c r="B109" s="3" t="s">
-        <v>603</v>
-      </c>
-      <c r="C109" s="3">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A110" s="3">
-        <v>110</v>
-      </c>
-      <c r="B110" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="C110" s="3">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A111" s="3">
-        <v>111</v>
-      </c>
-      <c r="B111" s="3" t="s">
-        <v>335</v>
-      </c>
-      <c r="C111" s="3">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A112" s="3">
-        <v>112</v>
-      </c>
-      <c r="B112" s="3" t="s">
-        <v>625</v>
-      </c>
-      <c r="C112" s="3">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A113" s="3">
-        <v>113</v>
-      </c>
-      <c r="B113" s="3" t="s">
-        <v>784</v>
-      </c>
-      <c r="C113" s="3">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A114" s="3">
-        <v>114</v>
-      </c>
-      <c r="B114" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C114" s="3">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A115" s="3">
-        <v>115</v>
-      </c>
-      <c r="B115" s="3" t="s">
-        <v>785</v>
-      </c>
-      <c r="C115" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A116" s="3">
-        <v>116</v>
-      </c>
-      <c r="B116" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="C116" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A117" s="3">
-        <v>117</v>
-      </c>
-      <c r="B117" s="3" t="s">
-        <v>786</v>
-      </c>
-      <c r="C117" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A118" s="3">
-        <v>118</v>
-      </c>
-      <c r="B118" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="C118" s="3">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A119" s="3">
-        <v>119</v>
-      </c>
-      <c r="B119" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="C119" s="3">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -45402,6 +45293,1329 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
+  <dimension ref="A1:C119"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="8.83203125" style="3" customWidth="1"/>
+    <col min="3" max="16384" width="8.83203125" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="3">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="3">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C4" s="3">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="3">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C5" s="3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="3">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C6" s="3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>7</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>8</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="3">
+        <v>10</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="3">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
+        <v>11</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="3">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="3">
+        <v>12</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C12" s="3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="3">
+        <v>13</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C13" s="3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="3">
+        <v>14</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="3">
+        <v>15</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="3">
+        <v>16</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C16" s="3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="3">
+        <v>17</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="3">
+        <v>18</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="C18" s="3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="3">
+        <v>19</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C19" s="3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="3">
+        <v>20</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C20" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="3">
+        <v>21</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="3">
+        <v>22</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="C22" s="3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="3">
+        <v>23</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" s="3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="3">
+        <v>24</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C24" s="3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>25</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="3">
+        <v>26</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="3">
+        <v>27</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C27" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="3">
+        <v>28</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="3">
+        <v>29</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C29" s="3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="3">
+        <v>30</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C30" s="3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="3">
+        <v>31</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C31" s="3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="3">
+        <v>32</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C32" s="3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="3">
+        <v>33</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="3">
+        <v>34</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C34" s="3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="3">
+        <v>35</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C35" s="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="3">
+        <v>36</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C36" s="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="3">
+        <v>37</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="C37" s="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="3">
+        <v>38</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C38" s="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="3">
+        <v>39</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="C39" s="3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="3">
+        <v>40</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C40" s="3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" s="3">
+        <v>41</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="C41" s="3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="3">
+        <v>42</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="C42" s="3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" s="3">
+        <v>43</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>681</v>
+      </c>
+      <c r="C43" s="3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" s="3">
+        <v>44</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="C44" s="3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" s="3">
+        <v>45</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="C45" s="3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" s="3">
+        <v>46</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="C46" s="3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <v>47</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="C47" s="3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" s="3">
+        <v>48</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="C48" s="3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" s="3">
+        <v>49</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C49" s="3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" s="3">
+        <v>50</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C50" s="3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" s="3">
+        <v>51</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C51" s="3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" s="3">
+        <v>52</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="C52" s="3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" s="3">
+        <v>53</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="C53" s="3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" s="3">
+        <v>54</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="C54" s="3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" s="3">
+        <v>55</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C55" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" s="3">
+        <v>56</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>631</v>
+      </c>
+      <c r="C56" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" s="3">
+        <v>57</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C57" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="3">
+        <v>58</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C58" s="3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="3">
+        <v>59</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C59" s="3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="3">
+        <v>60</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C60" s="3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="3">
+        <v>61</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C61" s="3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="3">
+        <v>62</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C62" s="3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="3">
+        <v>63</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C63" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="3">
+        <v>64</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C64" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="3">
+        <v>65</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="C65" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="3">
+        <v>66</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="C66" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="3">
+        <v>67</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C67" s="3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="3">
+        <v>68</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C68" s="3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="3">
+        <v>69</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C69" s="3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="3">
+        <v>70</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C70" s="3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="3">
+        <v>71</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C71" s="3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="3">
+        <v>72</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C72" s="3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="3">
+        <v>73</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C73" s="3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74" s="3">
+        <v>74</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C74" s="3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75" s="3">
+        <v>75</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>781</v>
+      </c>
+      <c r="C75" s="3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76" s="3">
+        <v>76</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>714</v>
+      </c>
+      <c r="C76" s="3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77" s="3">
+        <v>77</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>782</v>
+      </c>
+      <c r="C77" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A78" s="3">
+        <v>78</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="C78" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A79" s="3">
+        <v>79</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C79" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A80" s="3">
+        <v>80</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="C80" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A81" s="3">
+        <v>81</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C81" s="3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A82" s="3">
+        <v>82</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="C82" s="3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A83" s="3">
+        <v>83</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>744</v>
+      </c>
+      <c r="C83" s="3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A84" s="3">
+        <v>84</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>621</v>
+      </c>
+      <c r="C84" s="3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A85" s="3">
+        <v>85</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C85" s="3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A86" s="3">
+        <v>86</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="C86" s="3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A87" s="3">
+        <v>87</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="C87" s="3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A88" s="3">
+        <v>88</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C88" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A89" s="3">
+        <v>89</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>644</v>
+      </c>
+      <c r="C89" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90" s="3">
+        <v>90</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>705</v>
+      </c>
+      <c r="C90" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91" s="3">
+        <v>91</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C91" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A92" s="3">
+        <v>92</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="C92" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A93" s="3">
+        <v>93</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="C93" s="3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A94" s="3">
+        <v>94</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>783</v>
+      </c>
+      <c r="C94" s="3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A95" s="3">
+        <v>95</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="C95" s="3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A96" s="3">
+        <v>96</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C96" s="3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A97" s="3">
+        <v>97</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="C97" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A98" s="3">
+        <v>98</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="C98" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A99" s="3">
+        <v>99</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C99" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A100" s="3">
+        <v>100</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>778</v>
+      </c>
+      <c r="C100" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A101" s="3">
+        <v>101</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C101" s="3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A102" s="3">
+        <v>102</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C102" s="3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A103" s="3">
+        <v>103</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C103" s="3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A104" s="3">
+        <v>104</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>607</v>
+      </c>
+      <c r="C104" s="3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A105" s="3">
+        <v>105</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C105" s="3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A106" s="3">
+        <v>106</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="C106" s="3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A107" s="3">
+        <v>107</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="C107" s="3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A108" s="3">
+        <v>108</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="C108" s="3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A109" s="3">
+        <v>109</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>603</v>
+      </c>
+      <c r="C109" s="3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A110" s="3">
+        <v>110</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C110" s="3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A111" s="3">
+        <v>111</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="C111" s="3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A112" s="3">
+        <v>112</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="C112" s="3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A113" s="3">
+        <v>113</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="C113" s="3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A114" s="3">
+        <v>114</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C114" s="3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A115" s="3">
+        <v>115</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>785</v>
+      </c>
+      <c r="C115" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A116" s="3">
+        <v>116</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C116" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A117" s="3">
+        <v>117</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>786</v>
+      </c>
+      <c r="C117" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A118" s="3">
+        <v>118</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="C118" s="3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A119" s="3">
+        <v>119</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>787</v>
+      </c>
+      <c r="C119" s="3">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
   <dimension ref="A1:C82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -46317,7 +47531,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
   <dimension ref="A1:C173"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -48234,7 +49448,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <dimension ref="A1:C200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -50448,7 +51662,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
   <dimension ref="A1:C118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -51760,7 +52974,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2800-000000000000}">
   <dimension ref="A1:C79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>